<commit_message>
docs(shakeout): merge Daily Shakeout test cases into New_Testcase.xlsx
</commit_message>
<xml_diff>
--- a/Automation/tests/New_Testcase.xlsx
+++ b/Automation/tests/New_Testcase.xlsx
@@ -1,28 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A19F34D0-A453-4053-B459-286BAE18CD24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500"/>
   </bookViews>
   <sheets>
-    <sheet name="Step case and steps" sheetId="1" r:id="rId1"/>
-    <sheet name="Test data" sheetId="2" r:id="rId2"/>
-    <sheet name="Console Errors" sheetId="3" r:id="rId3"/>
-    <sheet name="Jira Tracker" sheetId="4" r:id="rId4"/>
-    <sheet name="API Test Cases" sheetId="5" r:id="rId5"/>
+    <sheet sheetId="1" name="Step case and steps" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Test data" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Console Errors" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Jira Tracker" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="API Test Cases" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="Daily Shakeout" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Step case and steps'!$A$2:$I$2</definedName>
+    <definedName name="_xlnm._FilterDatabase">'Step case and steps'!$A$2:$I$2</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5238" uniqueCount="629">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5421" uniqueCount="722">
   <si>
     <t>Test case</t>
   </si>
@@ -1909,27 +1909,368 @@
   </si>
   <si>
     <t>PATCH /api/v1/users/me/password with valid auth and data → 200</t>
+  </si>
+  <si>
+    <t>S.No</t>
+  </si>
+  <si>
+    <t>Test Group</t>
+  </si>
+  <si>
+    <t>Test File</t>
+  </si>
+  <si>
+    <t>Steps</t>
+  </si>
+  <si>
+    <t>Expected Result</t>
+  </si>
+  <si>
+    <t>Env</t>
+  </si>
+  <si>
+    <t>Run for Smoketest</t>
+  </si>
+  <si>
+    <t>01-tg1-login-health.spec.ts</t>
+  </si>
+  <si>
+    <t>Login page loads — HTTP 200, no server errors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to /login
+2. Verify HTTP status &lt; 400
+3. Verify email input field is visible</t>
+  </si>
+  <si>
+    <t>Login page renders with email input</t>
+  </si>
+  <si>
+    <t>POC + Prod</t>
+  </si>
+  <si>
+    <t>Health endpoint — API backend is alive</t>
+  </si>
+  <si>
+    <t>1. GET /api/v1/health</t>
+  </si>
+  <si>
+    <t>HTTP 200 response</t>
+  </si>
+  <si>
+    <t>Auth login — valid credentials return access token</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. POST /auth/login with admin credentials
+2. Verify response has accessToken
+3. Verify user.email matches input</t>
+  </si>
+  <si>
+    <t>HTTP 200 + valid JWT token returned</t>
+  </si>
+  <si>
+    <t>Auth login — invalid credentials return 401</t>
+  </si>
+  <si>
+    <t>1. POST /auth/login with invalid email/password</t>
+  </si>
+  <si>
+    <t>HTTP 401 Unauthorized</t>
+  </si>
+  <si>
+    <t>02-tg2-tg3-tg4-navigation.spec.ts</t>
+  </si>
+  <si>
+    <t>Admin login — Create new button and Admin dropdown visible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Login as admin
+2. Dismiss onboarding wizard
+3. Verify "Create new" button visible
+4. Verify Admin button in sidebar</t>
+  </si>
+  <si>
+    <t>Both Create new and Admin dropdown are visible</t>
+  </si>
+  <si>
+    <t>Workspace pages load — Audit Groups, Pulse, Policies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate /audit-groups → verify no error
+2. Navigate /pulse → verify "active audit" text
+3. Navigate /policies → verify "create policy" button</t>
+  </si>
+  <si>
+    <t>All 3 workspace pages load without errors</t>
+  </si>
+  <si>
+    <t>Contributor login — Admin, Policies, Pulse, Integrations NOT visible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Login as contributor
+2. Verify Admin button NOT visible
+3. Verify /policies link NOT visible
+4. Verify /pulse link NOT visible
+5. Verify /integrations link NOT visible</t>
+  </si>
+  <si>
+    <t>All 4 restricted tabs hidden for contributor</t>
+  </si>
+  <si>
+    <t>All Admin sub-tabs load without errors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Login as admin
+2. /admin → verify Add user button
+3. /admin/roles → verify Create role button
+4. /admin/integrations → no error
+5. /admin/features → no error
+6. /admin/activity → no error
+7. /admin/organization → no error</t>
+  </si>
+  <si>
+    <t>All 6 admin sub-pages load without errors</t>
+  </si>
+  <si>
+    <t>03-tg6-audit-lifecycle.spec.ts</t>
+  </si>
+  <si>
+    <t>Step 1-2: Audit tiles are visible on home page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Login as admin
+2. Navigate to /
+3. Verify at least one audit tile link exists</t>
+  </si>
+  <si>
+    <t>At least 1 audit tile visible</t>
+  </si>
+  <si>
+    <t>Step 3: Search box is visible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to /
+2. Verify search input with placeholder "Search" is visible</t>
+  </si>
+  <si>
+    <t>Search box is displayed</t>
+  </si>
+  <si>
+    <t>Step 4: Search by framework name filters matching audits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Type "SOC" in search box
+2. Wait 2 seconds
+3. Verify audit tiles filter (count &gt;= 0)</t>
+  </si>
+  <si>
+    <t>Search filters audits by framework name</t>
+  </si>
+  <si>
+    <t>Step 5: Search by audit name filters matching audits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Get first audit tile text
+2. Type first 5 chars in search
+3. Verify page still renders main content</t>
+  </si>
+  <si>
+    <t>Search filters by partial audit name</t>
+  </si>
+  <si>
+    <t>Step 6: Click audit tile — shows 5 tabs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click first audit tile
+2. Wait for /audit/ URL
+3. Verify &gt;= 5 tabs visible
+4. Verify: Dashboard, Workspace, Internal Audit, Document, Action Plan</t>
+  </si>
+  <si>
+    <t>Audit detail page shows all 5 tabs</t>
+  </si>
+  <si>
+    <t>MC</t>
+  </si>
+  <si>
+    <t>04-mc-availability.spec.ts</t>
+  </si>
+  <si>
+    <t>Mission Control — app is reachable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. GET {mcUrl}/login
+2. Verify HTTP status &lt; 500</t>
+  </si>
+  <si>
+    <t>MC responds without server error</t>
+  </si>
+  <si>
+    <t>Mission Control — page renders login form</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open {mcUrl}/login in browser
+2. Verify email input field is visible</t>
+  </si>
+  <si>
+    <t>MC login form renders</t>
+  </si>
+  <si>
+    <t>Audit Portal</t>
+  </si>
+  <si>
+    <t>05-audit-availability.spec.ts</t>
+  </si>
+  <si>
+    <t>Audit Portal — app is reachable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. GET {auditUrl}/login
+2. Verify HTTP status &lt; 500
+(Skipped on Prod — not ready)</t>
+  </si>
+  <si>
+    <t>Audit Portal responds without error</t>
+  </si>
+  <si>
+    <t>POC only</t>
+  </si>
+  <si>
+    <t>Audit Portal — page renders login form</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open {auditUrl}/login in browser
+2. Verify email input visible
+(Skipped on Prod — not ready)</t>
+  </si>
+  <si>
+    <t>Audit Portal login form renders</t>
+  </si>
+  <si>
+    <t>API</t>
+  </si>
+  <si>
+    <t>06-api-endpoints.spec.ts</t>
+  </si>
+  <si>
+    <t>Auth — obtain token for API tests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. POST /auth/login with admin creds
+2. Store accessToken</t>
+  </si>
+  <si>
+    <t>Token obtained successfully</t>
+  </si>
+  <si>
+    <t>GET /users/me — returns current user profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. GET /users/me with Bearer token
+2. Verify has id, email, roles</t>
+  </si>
+  <si>
+    <t>HTTP 200 + user profile</t>
+  </si>
+  <si>
+    <t>GET /frameworks — returns list with required fields</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. GET /frameworks
+2. Verify array length &gt; 0
+3. Verify each has id, name, sourceType</t>
+  </si>
+  <si>
+    <t>HTTP 200 + non-empty framework list</t>
+  </si>
+  <si>
+    <t>GET /audits — returns audit list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. GET /audits
+2. Verify HTTP 200 + returns array</t>
+  </si>
+  <si>
+    <t>HTTP 200 + audit array</t>
+  </si>
+  <si>
+    <t>GET /users — returns user list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. GET /users
+2. Verify length &gt; 0
+3. Verify has id, email</t>
+  </si>
+  <si>
+    <t>HTTP 200 + user list</t>
+  </si>
+  <si>
+    <t>GET /policies — returns policy list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. GET /policies
+2. Verify HTTP 200</t>
+  </si>
+  <si>
+    <t>HTTP 200</t>
+  </si>
+  <si>
+    <t>GET /business-units — returns list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. GET /business-units
+2. Verify status &lt; 500 (403 = alive but restricted)</t>
+  </si>
+  <si>
+    <t>No server error (200 or 403)</t>
+  </si>
+  <si>
+    <t>API response time — no endpoint exceeds 5s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Hit /health, /frameworks, /audits, /users, /policies
+2. Measure response time
+3. Verify none &gt; 5000ms</t>
+  </si>
+  <si>
+    <t>All endpoints respond within 5 seconds</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4472C4"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -1944,15 +2285,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -2285,16 +2633,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J65"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="134" customWidth="1"/>
-    <col min="5" max="5" width="42.25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="42.25" customWidth="1"/>
+    <col min="6" max="6" width="19.33203125" customWidth="1"/>
+    <col min="7" max="7" width="22.33203125" customWidth="1"/>
+    <col min="8" max="8" width="20.5" customWidth="1"/>
+    <col min="9" max="9" width="12.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2329,7 +2677,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -2337,7 +2685,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -2427,7 +2775,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -2467,7 +2815,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>30</v>
       </c>
@@ -2624,7 +2972,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>51</v>
       </c>
@@ -2667,7 +3015,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>54</v>
       </c>
@@ -2693,7 +3041,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>54</v>
       </c>
@@ -2719,7 +3067,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>54</v>
       </c>
@@ -2745,7 +3093,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>54</v>
       </c>
@@ -2771,7 +3119,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>62</v>
       </c>
@@ -2837,7 +3185,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>64</v>
       </c>
@@ -2892,7 +3240,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>64</v>
       </c>
@@ -2918,7 +3266,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>64</v>
       </c>
@@ -2944,7 +3292,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>75</v>
       </c>
@@ -3068,7 +3416,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>77</v>
       </c>
@@ -3094,7 +3442,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>77</v>
       </c>
@@ -3120,7 +3468,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>77</v>
       </c>
@@ -3175,7 +3523,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>77</v>
       </c>
@@ -3201,7 +3549,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>77</v>
       </c>
@@ -3256,7 +3604,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>77</v>
       </c>
@@ -3282,7 +3630,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>77</v>
       </c>
@@ -3308,7 +3656,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>77</v>
       </c>
@@ -3334,7 +3682,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>77</v>
       </c>
@@ -3360,7 +3708,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>77</v>
       </c>
@@ -3444,7 +3792,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>116</v>
       </c>
@@ -3458,7 +3806,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>118</v>
       </c>
@@ -3600,7 +3948,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>118</v>
       </c>
@@ -3626,7 +3974,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>130</v>
       </c>
@@ -3652,7 +4000,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>130</v>
       </c>
@@ -3678,7 +4026,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>130</v>
       </c>
@@ -3704,7 +4052,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>130</v>
       </c>
@@ -3730,7 +4078,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>130</v>
       </c>
@@ -3843,7 +4191,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>145</v>
       </c>
@@ -3869,7 +4217,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>147</v>
       </c>
@@ -3895,7 +4243,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>149</v>
       </c>
@@ -3986,16 +4334,13 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:J44 A65:J65 A45:E64 G45:J56 H64:J64 H57:J57 H58:J58 H59:J59 H60:J60 H61:J61 H62:J62 H63:J63" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -4072,23 +4417,20 @@
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
-    <hyperlink ref="B4" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
-    <hyperlink ref="B5" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
-    <hyperlink ref="B6" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
-    <hyperlink ref="B7" r:id="rId5" xr:uid="{00000000-0004-0000-0100-000004000000}"/>
+    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="B4" r:id="rId2"/>
+    <hyperlink ref="B5" r:id="rId3"/>
+    <hyperlink ref="B6" r:id="rId4"/>
+    <hyperlink ref="B7" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:C7" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H32"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -4924,16 +5266,13 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:H32" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K4"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -5077,16 +5416,13 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:K4" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J489"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -20738,8 +21074,702 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:J489" numberStoredAsText="1"/>
-  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H26"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="38" customWidth="1"/>
+    <col min="4" max="4" width="65" customWidth="1"/>
+    <col min="5" max="5" width="100" style="2" customWidth="1"/>
+    <col min="6" max="6" width="50" style="2" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>629</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>630</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>631</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>632</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>633</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>636</v>
+      </c>
+      <c r="D2" t="s">
+        <v>637</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="G2" t="s">
+        <v>640</v>
+      </c>
+      <c r="H2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>636</v>
+      </c>
+      <c r="D3" t="s">
+        <v>641</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>642</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>643</v>
+      </c>
+      <c r="G3" t="s">
+        <v>640</v>
+      </c>
+      <c r="H3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>636</v>
+      </c>
+      <c r="D4" t="s">
+        <v>644</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>645</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>646</v>
+      </c>
+      <c r="G4" t="s">
+        <v>640</v>
+      </c>
+      <c r="H4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>636</v>
+      </c>
+      <c r="D5" t="s">
+        <v>647</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>648</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>649</v>
+      </c>
+      <c r="G5" t="s">
+        <v>640</v>
+      </c>
+      <c r="H5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" t="s">
+        <v>650</v>
+      </c>
+      <c r="D6" t="s">
+        <v>651</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>653</v>
+      </c>
+      <c r="G6" t="s">
+        <v>640</v>
+      </c>
+      <c r="H6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" t="s">
+        <v>650</v>
+      </c>
+      <c r="D7" t="s">
+        <v>654</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>655</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="G7" t="s">
+        <v>640</v>
+      </c>
+      <c r="H7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" t="s">
+        <v>650</v>
+      </c>
+      <c r="D8" t="s">
+        <v>657</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>659</v>
+      </c>
+      <c r="G8" t="s">
+        <v>640</v>
+      </c>
+      <c r="H8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" t="s">
+        <v>650</v>
+      </c>
+      <c r="D9" t="s">
+        <v>660</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>662</v>
+      </c>
+      <c r="G9" t="s">
+        <v>640</v>
+      </c>
+      <c r="H9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>120</v>
+      </c>
+      <c r="C10" t="s">
+        <v>663</v>
+      </c>
+      <c r="D10" t="s">
+        <v>664</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>665</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>666</v>
+      </c>
+      <c r="G10" t="s">
+        <v>640</v>
+      </c>
+      <c r="H10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>120</v>
+      </c>
+      <c r="C11" t="s">
+        <v>663</v>
+      </c>
+      <c r="D11" t="s">
+        <v>667</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>668</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="G11" t="s">
+        <v>640</v>
+      </c>
+      <c r="H11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>120</v>
+      </c>
+      <c r="C12" t="s">
+        <v>663</v>
+      </c>
+      <c r="D12" t="s">
+        <v>670</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>671</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="G12" t="s">
+        <v>640</v>
+      </c>
+      <c r="H12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>120</v>
+      </c>
+      <c r="C13" t="s">
+        <v>663</v>
+      </c>
+      <c r="D13" t="s">
+        <v>673</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>674</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>675</v>
+      </c>
+      <c r="G13" t="s">
+        <v>640</v>
+      </c>
+      <c r="H13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>120</v>
+      </c>
+      <c r="C14" t="s">
+        <v>663</v>
+      </c>
+      <c r="D14" t="s">
+        <v>676</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>677</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>678</v>
+      </c>
+      <c r="G14" t="s">
+        <v>640</v>
+      </c>
+      <c r="H14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>679</v>
+      </c>
+      <c r="C15" t="s">
+        <v>680</v>
+      </c>
+      <c r="D15" t="s">
+        <v>681</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>682</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="G15" t="s">
+        <v>640</v>
+      </c>
+      <c r="H15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>679</v>
+      </c>
+      <c r="C16" t="s">
+        <v>680</v>
+      </c>
+      <c r="D16" t="s">
+        <v>684</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>685</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>686</v>
+      </c>
+      <c r="G16" t="s">
+        <v>640</v>
+      </c>
+      <c r="H16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>687</v>
+      </c>
+      <c r="C17" t="s">
+        <v>688</v>
+      </c>
+      <c r="D17" t="s">
+        <v>689</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>690</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>691</v>
+      </c>
+      <c r="G17" t="s">
+        <v>692</v>
+      </c>
+      <c r="H17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>687</v>
+      </c>
+      <c r="C18" t="s">
+        <v>688</v>
+      </c>
+      <c r="D18" t="s">
+        <v>693</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>695</v>
+      </c>
+      <c r="G18" t="s">
+        <v>692</v>
+      </c>
+      <c r="H18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>696</v>
+      </c>
+      <c r="C19" t="s">
+        <v>697</v>
+      </c>
+      <c r="D19" t="s">
+        <v>698</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>699</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>700</v>
+      </c>
+      <c r="G19" t="s">
+        <v>640</v>
+      </c>
+      <c r="H19" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>696</v>
+      </c>
+      <c r="C20" t="s">
+        <v>697</v>
+      </c>
+      <c r="D20" t="s">
+        <v>701</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>702</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>703</v>
+      </c>
+      <c r="G20" t="s">
+        <v>640</v>
+      </c>
+      <c r="H20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>696</v>
+      </c>
+      <c r="C21" t="s">
+        <v>697</v>
+      </c>
+      <c r="D21" t="s">
+        <v>704</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>706</v>
+      </c>
+      <c r="G21" t="s">
+        <v>640</v>
+      </c>
+      <c r="H21" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>696</v>
+      </c>
+      <c r="C22" t="s">
+        <v>697</v>
+      </c>
+      <c r="D22" t="s">
+        <v>707</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>708</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>709</v>
+      </c>
+      <c r="G22" t="s">
+        <v>640</v>
+      </c>
+      <c r="H22" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>696</v>
+      </c>
+      <c r="C23" t="s">
+        <v>697</v>
+      </c>
+      <c r="D23" t="s">
+        <v>710</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>711</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="G23" t="s">
+        <v>640</v>
+      </c>
+      <c r="H23" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>696</v>
+      </c>
+      <c r="C24" t="s">
+        <v>697</v>
+      </c>
+      <c r="D24" t="s">
+        <v>713</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>714</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>715</v>
+      </c>
+      <c r="G24" t="s">
+        <v>640</v>
+      </c>
+      <c r="H24" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>696</v>
+      </c>
+      <c r="C25" t="s">
+        <v>697</v>
+      </c>
+      <c r="D25" t="s">
+        <v>716</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>717</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>718</v>
+      </c>
+      <c r="G25" t="s">
+        <v>640</v>
+      </c>
+      <c r="H25" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>696</v>
+      </c>
+      <c r="C26" t="s">
+        <v>697</v>
+      </c>
+      <c r="D26" t="s">
+        <v>719</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>720</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>721</v>
+      </c>
+      <c r="G26" t="s">
+        <v>640</v>
+      </c>
+      <c r="H26" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
config: disable Jira ticket creation in Configuration sheet
</commit_message>
<xml_diff>
--- a/Automation/tests/New_Testcase.xlsx
+++ b/Automation/tests/New_Testcase.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15AA6BA3-5AB2-4BAF-98F9-F82FBD6AF2A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73C4A165-88C2-43CF-A36D-9B5F90397103}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="727" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="727" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Regression" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5562" uniqueCount="696">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5559" uniqueCount="696">
   <si>
     <t>Test case</t>
   </si>
@@ -2502,7 +2502,7 @@
   <dimension ref="A1:I71"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="49.58203125" customWidth="1"/>
+    <col min="2" max="2" width="86.9140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
@@ -22008,7 +22008,7 @@
         <v>685</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="C4" t="s">
         <v>686</v>
@@ -22080,7 +22080,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:C1 A3:C5 A2 C2 A7:C10 A6 C6" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:C1 A3:C3 A2 C2 A7:C10 A6 C6 A5:C5 A4 C4" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
config: update Configuration sheet — remove email recipient
</commit_message>
<xml_diff>
--- a/Automation/tests/New_Testcase.xlsx
+++ b/Automation/tests/New_Testcase.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73C4A165-88C2-43CF-A36D-9B5F90397103}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40D73947-77AE-48DD-B85E-1DEA1B513712}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="727" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5559" uniqueCount="696">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5559" uniqueCount="695">
   <si>
     <t>Test case</t>
   </si>
@@ -2109,9 +2109,6 @@
   </si>
   <si>
     <t>• Push to GitHub for CI runs to pick up changes.</t>
-  </si>
-  <si>
-    <t>keerthi@quantarra.io, deepak@quantarra.io</t>
   </si>
 </sst>
 </file>
@@ -4294,7 +4291,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:I56 A71:I71 A65:C65 H65:I65 A66:C66 H66:I66 A67:C67 H67:I67 A68:C68 H68:I68 A69:C69 H69:I69 A70:C70 H70:I70 A64:F64 A57:F57 H57:I57 A58:F58 H58:I58 A59:F59 H59:I59 A60:F60 H60:I60 A61:F61 H61:I61 A62:F62 H62:I62 A63:F63 H63:I63 H64:I64" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:I56 A71:I71 A65:C65 H65:I65 A66:C66 H66:I66 A67:C67 H67:I67 A68:C68 H68:I68 A69:C69 H69:I69 A70:C70 H70:I70 A64:F64 A57 H57:I57 A58:F58 H58:I58 A59:F59 H59:I59 A60:F60 H60:I60 A61:F61 H61:I61 A62:F62 H62:I62 A63:F63 H63:I63 H64:I64 C57:F57" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -22029,8 +22026,8 @@
       <c r="A6" t="s">
         <v>690</v>
       </c>
-      <c r="B6" t="s">
-        <v>695</v>
+      <c r="B6" s="1" t="s">
+        <v>631</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
@@ -22078,6 +22075,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B6" r:id="rId1" xr:uid="{6794E79B-E8D6-4D28-8342-139A5ED5576A}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError sqref="A1:C1 A3:C3 A2 C2 A7:C10 A6 C6 A5:C5 A4 C4" numberStoredAsText="1"/>

</xml_diff>

<commit_message>
test(regression): refine TG-3 Scenario 3 TC-1 and TC-7
TC-1: assert the contributor logs in specifically as 'Matrix Contributor'
(was a generic /contributor/ text match).

TC-7: validate audit tiles against the expected framework. Locally defaults to
SOC 2 Type 2; in GitHub Actions reads the workflow 'framework' input via the
FRAMEWORK_TYPE env var (falls back to SOC 2 Type 2 when N/A/unset).

Includes the Scenario 3 Excel description updates. Verified passing on staging.
</commit_message>
<xml_diff>
--- a/Automation/tests/New_Testcase.xlsx
+++ b/Automation/tests/New_Testcase.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_D688307FDBA934CE52A31ED8FB17F8A4534B0E35" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6F6E263-7F90-46D0-BDB3-D8E14121EC34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Regression" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
test(regression): refine TG-3 Scenario 3 TC-1 and TC-7 (#5)
TC-1: assert the contributor logs in specifically as 'Matrix Contributor'
(was a generic /contributor/ text match).

TC-7: validate audit tiles against the expected framework. Locally defaults to
SOC 2 Type 2; in GitHub Actions reads the workflow 'framework' input via the
FRAMEWORK_TYPE env var (falls back to SOC 2 Type 2 when N/A/unset).

Includes the Scenario 3 Excel description updates. Verified passing on staging.
</commit_message>
<xml_diff>
--- a/Automation/tests/New_Testcase.xlsx
+++ b/Automation/tests/New_Testcase.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_D688307FDBA934CE52A31ED8FB17F8A4534B0E35" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6F6E263-7F90-46D0-BDB3-D8E14121EC34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Regression" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
test(regression): track PRJAT-1260 in Excel Jira Tracker
Add PRJAT-1260 (Internal Audit filter button missing active-filter badge) to the
Jira Tracker sheet of New_Testcase.xlsx, linked to TG-7 Scenario 7 TC-11b.
</commit_message>
<xml_diff>
--- a/Automation/tests/New_Testcase.xlsx
+++ b/Automation/tests/New_Testcase.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5770" uniqueCount="743">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5781" uniqueCount="749">
   <si>
     <t>Test case</t>
   </si>
@@ -2198,6 +2198,24 @@
   </si>
   <si>
     <t>TG-1 to TG-7 (all)</t>
+  </si>
+  <si>
+    <t>PRJAT-1260</t>
+  </si>
+  <si>
+    <t>[QA] Internal Audit tab: filter button does not show active-filter count badge</t>
+  </si>
+  <si>
+    <t>qa-block, staging</t>
+  </si>
+  <si>
+    <t>To Do</t>
+  </si>
+  <si>
+    <t>TG-7 Scenario 7 TC-11b</t>
+  </si>
+  <si>
+    <t>2026-08-30</t>
   </si>
   <si>
     <t>Setting</t>
@@ -2684,7 +2702,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -3160,7 +3178,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>58</v>
       </c>
@@ -3333,7 +3351,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="28" ht="14.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>70</v>
       </c>
@@ -3833,7 +3851,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="47" ht="14.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" ht="14.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>109</v>
       </c>
@@ -22621,7 +22639,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="15.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="9.26953125" customWidth="1"/>
@@ -22770,6 +22788,41 @@
         <v>18</v>
       </c>
       <c r="K4" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>725</v>
+      </c>
+      <c r="B5" t="s">
+        <v>726</v>
+      </c>
+      <c r="C5" t="s">
+        <v>709</v>
+      </c>
+      <c r="D5" t="s">
+        <v>710</v>
+      </c>
+      <c r="E5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F5" t="s">
+        <v>155</v>
+      </c>
+      <c r="G5" t="s">
+        <v>727</v>
+      </c>
+      <c r="H5" t="s">
+        <v>728</v>
+      </c>
+      <c r="I5" t="s">
+        <v>729</v>
+      </c>
+      <c r="J5" t="s">
+        <v>730</v>
+      </c>
+      <c r="K5" t="s">
         <v>716</v>
       </c>
     </row>
@@ -22789,70 +22842,70 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>725</v>
+        <v>731</v>
       </c>
       <c r="B1" t="s">
-        <v>726</v>
+        <v>732</v>
       </c>
       <c r="C1" t="s">
-        <v>727</v>
+        <v>733</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>728</v>
+        <v>734</v>
       </c>
       <c r="B2" t="s">
         <v>36</v>
       </c>
       <c r="C2" t="s">
-        <v>729</v>
+        <v>735</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>730</v>
+        <v>736</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>731</v>
+        <v>737</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>732</v>
+        <v>738</v>
       </c>
       <c r="B4" t="s">
         <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>733</v>
+        <v>739</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>734</v>
+        <v>740</v>
       </c>
       <c r="B5" t="s">
-        <v>735</v>
+        <v>741</v>
       </c>
       <c r="C5" t="s">
-        <v>736</v>
+        <v>742</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>737</v>
+        <v>743</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>738</v>
+        <v>744</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>739</v>
+        <v>745</v>
       </c>
       <c r="B7" t="s">
         <v>155</v>
@@ -22863,7 +22916,7 @@
     </row>
     <row r="8" ht="15.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>740</v>
+        <v>746</v>
       </c>
       <c r="B8" t="s">
         <v>155</v>
@@ -22874,7 +22927,7 @@
     </row>
     <row r="9" ht="15.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>741</v>
+        <v>747</v>
       </c>
       <c r="B9" t="s">
         <v>155</v>
@@ -22885,7 +22938,7 @@
     </row>
     <row r="10" ht="15.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>742</v>
+        <v>748</v>
       </c>
       <c r="B10" t="s">
         <v>155</v>

</xml_diff>